<commit_message>
Renditions-Katalog LRA NDR aus aktualisierter renditions.xlsx (V1.1).
21 Formate inkl. Import-Skript und LRA-erweiterbare Struktur für weitere Landesrundfunkanstalten.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/renditions.xlsx
+++ b/renditions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lentzh/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC643AB0-317D-FE46-979B-C11701EF598B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF309ECB-0F4C-DD4C-BE90-2726A5CDFE36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3880" yWindow="2740" windowWidth="28240" windowHeight="17240" xr2:uid="{3CBA87E5-6815-1940-9170-18C0B1F3930C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="82">
   <si>
     <t>HEVC (WebL)</t>
   </si>
@@ -56,9 +56,6 @@
     <t>seit Mai 2022</t>
   </si>
   <si>
-    <t>HEVC SDR 540</t>
-  </si>
-  <si>
     <t>HEVC (WebXL)</t>
   </si>
   <si>
@@ -68,9 +65,6 @@
     <t>1280x720</t>
   </si>
   <si>
-    <t>HEVC SDR 720</t>
-  </si>
-  <si>
     <t>HEVC (Full-HD 1080p)</t>
   </si>
   <si>
@@ -80,9 +74,6 @@
     <t>1920x1080</t>
   </si>
   <si>
-    <t>HEVC SDR 1080</t>
-  </si>
-  <si>
     <t>HEVC-HDR (Full-HD 1080p)</t>
   </si>
   <si>
@@ -92,9 +83,6 @@
     <t>nur bei UHD-HDR</t>
   </si>
   <si>
-    <t>HEVC HDR 1080</t>
-  </si>
-  <si>
     <t>HEVC-HDR (1440)</t>
   </si>
   <si>
@@ -104,9 +92,6 @@
     <t>2560x1440</t>
   </si>
   <si>
-    <t>HEVC HDR 1440</t>
-  </si>
-  <si>
     <t>HEVC-HDR (2160)</t>
   </si>
   <si>
@@ -116,9 +101,6 @@
     <t>3180x2160</t>
   </si>
   <si>
-    <t>HEVC HDR 2160</t>
-  </si>
-  <si>
     <t>VP9 (WebL)</t>
   </si>
   <si>
@@ -128,30 +110,18 @@
     <t>VP9</t>
   </si>
   <si>
-    <t>ab Mai 2022, 2024 weggefallen</t>
-  </si>
-  <si>
-    <t>VP9 540</t>
-  </si>
-  <si>
     <t>VP9 (WebXL)</t>
   </si>
   <si>
     <t>.hd.vp9.mp4</t>
   </si>
   <si>
-    <t>VP9 720</t>
-  </si>
-  <si>
     <t>VP9 (Full-HD 1080p)</t>
   </si>
   <si>
     <t>.1080.vp9.mp4</t>
   </si>
   <si>
-    <t>VP9 1080</t>
-  </si>
-  <si>
     <t>Format</t>
   </si>
   <si>
@@ -168,6 +138,153 @@
   </si>
   <si>
     <t>ARD-Bezeichnung</t>
+  </si>
+  <si>
+    <t>MP4 (nur Audio)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>.ao.mp4</t>
+  </si>
+  <si>
+    <t>Audio only</t>
+  </si>
+  <si>
+    <t>März 2013 bis Juni 2025</t>
+  </si>
+  <si>
+    <t>MP4 (WebM niedrig)</t>
+  </si>
+  <si>
+    <t>avc270</t>
+  </si>
+  <si>
+    <t>.mn.mp4</t>
+  </si>
+  <si>
+    <t>480x270</t>
+  </si>
+  <si>
+    <t>H.264</t>
+  </si>
+  <si>
+    <t>seit 12.11.2014</t>
+  </si>
+  <si>
+    <t>MP4 (WebL niedrig)</t>
+  </si>
+  <si>
+    <t>avc360</t>
+  </si>
+  <si>
+    <t>.ln.mp4</t>
+  </si>
+  <si>
+    <t>640x360</t>
+  </si>
+  <si>
+    <t>MP4 (WebL)</t>
+  </si>
+  <si>
+    <t>avc540</t>
+  </si>
+  <si>
+    <t>.hq.mp4</t>
+  </si>
+  <si>
+    <t>MP4 (WebXL)</t>
+  </si>
+  <si>
+    <t>avc720</t>
+  </si>
+  <si>
+    <t>.hd.mp4</t>
+  </si>
+  <si>
+    <t>seit März 2015</t>
+  </si>
+  <si>
+    <t>MP4 (Full-HD 1080p)</t>
+  </si>
+  <si>
+    <t>avc1080</t>
+  </si>
+  <si>
+    <t>.1080.mp4</t>
+  </si>
+  <si>
+    <t>hevcsdr540</t>
+  </si>
+  <si>
+    <t>hevcsdr720</t>
+  </si>
+  <si>
+    <t>hevcsdr1080</t>
+  </si>
+  <si>
+    <t>hevchdr1080</t>
+  </si>
+  <si>
+    <t>hevchdr1440</t>
+  </si>
+  <si>
+    <t>hevchdr2160</t>
+  </si>
+  <si>
+    <t>vp9sdr540</t>
+  </si>
+  <si>
+    <t>ab Mai 2022, später weg</t>
+  </si>
+  <si>
+    <t>vp9sdr720</t>
+  </si>
+  <si>
+    <t>vp9sdr1080</t>
+  </si>
+  <si>
+    <t>MP4 (WebS)</t>
+  </si>
+  <si>
+    <t>.lo.mp4</t>
+  </si>
+  <si>
+    <t>320x180</t>
+  </si>
+  <si>
+    <t>weggefallen 2021</t>
+  </si>
+  <si>
+    <t>MP4 (WebM)</t>
+  </si>
+  <si>
+    <t>.hi.mp4</t>
+  </si>
+  <si>
+    <t>512x288</t>
+  </si>
+  <si>
+    <t>MP4 (WebL+)</t>
+  </si>
+  <si>
+    <t>.lp.mp4</t>
+  </si>
+  <si>
+    <t>720x576</t>
+  </si>
+  <si>
+    <t>Flash LOW</t>
+  </si>
+  <si>
+    <t>nicht mehr im Einsatz</t>
+  </si>
+  <si>
+    <t>Flash HIGH</t>
+  </si>
+  <si>
+    <t>Flash (L)</t>
   </si>
 </sst>
 </file>
@@ -545,215 +662,455 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0032719A-A60F-624B-8BD5-EC95D889EC40}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>9</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>3</v>
+        <v>47</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>15</v>
+        <v>49</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>21</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>25</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="E8" s="1" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>36</v>
+      <c r="D11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" t="s">
+        <v>3</v>
+      </c>
+      <c r="F11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" t="s">
+        <v>2</v>
+      </c>
+      <c r="E14" t="s">
+        <v>22</v>
+      </c>
+      <c r="F14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" t="s">
+        <v>22</v>
+      </c>
+      <c r="F16" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>68</v>
+      </c>
+      <c r="B17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" t="s">
+        <v>69</v>
+      </c>
+      <c r="D17" t="s">
+        <v>70</v>
+      </c>
+      <c r="E17" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" t="s">
+        <v>74</v>
+      </c>
+      <c r="E18" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" t="s">
+        <v>76</v>
+      </c>
+      <c r="D19" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" t="s">
+        <v>42</v>
+      </c>
+      <c r="F19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" t="s">
+        <v>34</v>
+      </c>
+      <c r="E20" t="s">
+        <v>34</v>
+      </c>
+      <c r="F20" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C21" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" t="s">
+        <v>34</v>
+      </c>
+      <c r="F21" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>81</v>
+      </c>
+      <c r="B22" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" t="s">
+        <v>34</v>
+      </c>
+      <c r="E22" t="s">
+        <v>34</v>
+      </c>
+      <c r="F22" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>